<commit_message>
PLR changes, parallel running, VerifAI fixes
</commit_message>
<xml_diff>
--- a/Work/policy/runs_results.xlsx
+++ b/Work/policy/runs_results.xlsx
@@ -340,7 +340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="2">
@@ -976,79 +976,146 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>p0.75srandom1231</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>2026-03-19 16:04:42</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" t="n">
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
         <v>0.75</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="3" t="n">
         <v>500000</v>
       </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="n">
+      <c r="F9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="3" t="n">
         <v>0.0003</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="3" t="n">
         <v>0.99</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>ppo</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
+      <c r="J9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" s="3" t="n">
         <v>1000</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="3" t="n">
         <v>90.75461978470474</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="3" t="n">
         <v>67.21087769566853</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="3" t="n">
         <v>105.5231256599789</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9" s="3" t="n">
         <v>4735</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>[1.299442970534115, 0.9242650286220793, 1.12362822991094, 1.2748945868627855, 1.6202752034895118, 0.9170680932342907, 1.0201072426456201, 0.9642534362941488, 0.8072701805092369, 0.5609159351701812, 0.9678233917217578, 1.7334811947102606, 1.7676914621177064, 1.5720809593725253, 2.134607444298924, 1.69896858518717, 0.9549259757172103, 1.8970720085815072, 1.9045028621729911, 0.4223298392725542, 0.6144116388587104, 1.0755350444746086, 0.9434942669838087, 1.1478932057731281, 0.9917901305072447, 1.123726065857584, 0.8140326300759346, 1.6320755370337063, 0.7660029372253463, 1.4433193240537294, 1.42839304440737, 0.9435879973792397, 1.77273157364622, 1.0051758305041816, 1.9083960850451598, 0.7220606113508456, 1.5425301933112219, 1.264892445100116, 1.8599551395552445, 1.0690845877499988, 0.8838361280809942, 1.5322989383329726, 2.3200865002574558, 2.21199972926878, 2.1619543848183223, 1.9255052323668398, 2.9957726094552592, 1.598082524105154, 1.531941284357969, 1.5772595742604427, 2.7958132548435324, 1.7559270581393847, 2.0592679998986205, 2.169556987827566, 2.090051180412207, 2.5241927789621146, 2.41842523364496, 1.005990330547241, 2.587864946632372, 1.9916446084656094, 2.1420745221759336, 1.4717412872456626, 1.6788364816562233, 1.1163329112347178, 1.1991142142659823, 4.658984112602143, 2.8320328298721615, 1.8121696663329956, 1.0364848432841212, 2.1173328570753402, 1.6984131850005864, 3.192883580168828, 2.4373144774873494, 3.346645755333631, 2.7578949886061106, 2.0360609287274687, 1.8461853670753356, 3.052856451725161, 2.7993931213793637, 3.494914841008577, 2.759113098094694, 2.3017548959749754, 3.1171977091111085, 3.6810231150233492, 4.619928460747222, 3.5667772994135456, 3.9545364691012934, 4.076298953570684, 5.841213960836444, 3.0444496137186903, 2.74147665897301, 3.0887726791562065, 2.2995803215059802, 5.464667632164034, 2.9447450333020577, 2.848511933984197, 5.056221302023285, 2.1238336451619695, 2.961598592197947, 0.9410721917448974, 0.5861321405971411, 7.216585311510752, 4.550057394956193, 4.907005966508597, 3.9405928103713936, 4.468400186171093, 2.6911874337811947, 3.450271412860009, 10.278888293875436, 9.075979647623097, 10.138880394732407, 5.546919421690232, 6.2065600282047555, 3.21034984397617, 7.936157899447315, 7.491123073633773, 8.069769877808746, 7.232841282181162, 3.5887482282255627, 2.888365246648476, 10.786743935673542, 3.7619511935791605, 6.435663233816966, 2.8038027150367086, 2.8233766701463527, 8.371337503110404, 8.701802097648663, 6.1726510450125085, 4.096300127186816, 7.19595953070761, 6.181246667870635, 5.472704415874364, 5.40178329094836, 3.032963238591095, 5.733318519141863, 4.576923367053697, 3.242636096462202, 8.706060923532844, 4.628981324332906, 7.031795148903673, 5.880129710900626, 3.97398881104584, 4.806673616474275, 10.921002369947736, 11.681624793520074, 4.508476838581816, 3.5100627742450294, 5.51379635213494, 10.090697291325018, 12.058056212197506, 9.9908314629725, 11.237479098522604, 8.962754266622097, 5.220309289360509, 14.209785604010504, 13.112461710155273, 6.76548065867348, 10.172635606712115, 7.815447099577768, 10.567107283426541, 15.63120211948765, 7.288813994909898, 5.575236331354684, 7.151710807596903, 6.65880989052829, 7.159867008893823, 10.879692997776294, 10.86719739202091, 7.975367387473729, 11.895352777282424, 7.933462529678846, 9.712249874479976, 7.904015627242476, 8.754074343880367, 6.949429681135454, 17.906784996757278, 6.0004344438768085, 10.026678336623723, 11.778933040611353, 13.770251310248666, 11.80029407991272, 13.564801400455304, 11.359277104283803, 12.646557317027899, 21.832605588955204, 9.188918841871097, 14.801429478670476, 18.932181805175905, 10.731251602902164, 19.120734070468984, 17.968050909311884, 10.990621308299907, 21.307883371001836, 30.254815046247003, 13.144978882544214, 25.777699291413793, 22.653511617729148, 18.197408042207623, 25.238022268231674, 8.298627541631499, 11.661296820810257, 26.6192973746, 24.505684874658822, 16.343344628855057, 20.10972840384654, 11.498147796911756, 18.072441255806886, 17.609465571766403, 12.372107581496659, 5.849862558450214, 11.73460183313949, 16.067143787049694, 8.668139849995256, 16.325873433643906, 16.35767472596624, 15.644794461250413, 15.101797935069577, 17.303358025384977, 18.172283616935843, 12.907207651730774, 35.91410593211549, 34.099439979870354, 29.842391626015694, 27.39082855089487, 29.463036353103792, 30.342339414053683, 26.845745708298562, 30.825850002284003, 28.05168650288439, 10.041115534816372, 8.345935687349156, 35.66833891338598, 25.8309429329926, 21.40922381941743, 23.416587848916006, 19.72189977165321, 23.40460349409636, 19.992329230622104, 26.52940664586418, 35.048114882107186, 47.0587348504069, 12.08337474249311, 25.37563365747458, 15.560278380720254, 40.02340183230565, 15.957853910254531, 29.17840148808246, 15.064928491970697, 31.451800587661353, 14.334807526072645, 30.298159560260515, 23.79706781147562, 25.76000523558445, 24.57316271093351, 18.92885261319706, 32.577870277608355, 21.635417044369337, 55.760413073379084, 23.771610709843657, 56.135853069672876, 35.65713470102574, 41.19696921536475, 25.30401200753934, 24.27951311270446, 31.59182881422566, 41.215380068830285, 12.767232257793212, 38.47716104826322, 22.600710061763255, 28.516745749263862, 33.76497055255826, 28.446609057990052, 30.302115650917553, 20.111653673397452, 29.18497263683876, 38.396777999888066, 32.27378589388955, 34.1072567156578, 35.56105274406334, 43.21418394401639, 32.08118194018602, 35.677360708508814, 23.242435412936224, 18.803844115013597, 36.7081594654593, 47.861137111275845, 28.460216032366905, 23.245762727262456, 42.051589522575725, 33.536033651099146, 25.571953417028993, 35.28728973427017, 22.55760760582797, 12.61597535710013, 27.02940872914391, 21.142810075340893, 29.790871200381734, 42.42167692397592, 55.21033710153082, 15.005011721548874, 35.121056430249126, 12.00418733591321, 58.302904387434, 23.72907225941933, 25.462709265496155, 42.288669218723136, 37.801723134110354, 53.60879691874695, 40.74016150829339, 42.41352686964786, 25.979472242515005, 17.188698632380717, 26.967179770105076, 37.2927932719069, 37.962202810812414, 23.331371210546635, 33.202423733419096, 55.07157351668646, 33.34108036982655, 5.008622015050751, 4.781686705103314, 58.043948020606926, 32.54299680031296, 42.05576226150764, 21.630100695689357, 18.73174532074214, 44.370302745518096, 42.74449245568722, 26.913950793982508, 35.18956559164732, 52.79447466291084, 47.47302513703453, 42.64379930877753, 29.751311635286296, 25.444891622842704, 33.33100694771483, 24.39217784218832, 61.86070076869198, 19.73516946601583, 35.28982336929973, 34.47921236396627, 26.31612383074453, 43.08878644278531, 35.71311694857227, 28.085410134719247, 48.97843893419593, 17.764291945052, 28.018964556801727, 24.669251298521473, 24.882162949106316, 34.83112629767116, 20.099637744738438, 33.94063273933182, 37.53840134791584, 32.18902669059011, 33.04983223252823, 30.229604756872863, 54.23303133855073, 39.978895117583306, 58.390799781992136, 31.90827950502552, 27.70847005033227, 33.85649988481415, 59.85759187097741, 89.35282402329273, 36.49181857178372, 41.98771725152491, 39.05014678826906, 35.35678774925792, 35.33742770361992, 42.77880787199321, 40.40883582757039, 53.91140515627098, 35.80859845866236, 89.55826828487696, 81.01738979900892, 33.521531570272195, 44.68521111019893, 24.774762287078257, 18.607059137507253, 69.30792084784308, 30.447171737098177, 67.49404891521057, 68.11535912764712, 20.25884933981441, 50.5291185375236, 37.22663816181516, 30.140351173539084, 28.515699657377596, 36.63102628334285, 71.25457189425873, 33.51754611334671, 27.776267071453805, 27.909700294582755, 69.82621546020337, 32.60005619556792, 69.28532177194532, 75.4436640097749, 61.08661662204542, 73.81349441185161, 58.88649103076485, 30.78051680352343, 49.30931960941643, 31.111289834639635, 48.848150387487195, 72.8736276706957, 65.29718183181825, 29.965092230019973, 58.476544037222, 39.51843640906734, 56.391887192160354, 42.59871147975467, 51.25994764810019, 54.35930322945424, 75.61256635740808, 38.65966568440267, 53.0219012765528, 50.0925196038127, 24.310010914001865, 36.38825304315579, 32.57506197203899, 39.04948106333704, 39.24199559537596, 21.71751030913504, 37.758210440112926, 42.3625918558355, 35.860083192287966, 54.98544979018975, 36.1707360329646, 51.985885063531924, 48.9671987051987, 37.62487960936804, 67.89752043216663, 6.447781184602794, 8.581503219596332, 26.448416136966536, 35.95767820637758, 66.04162130071542, 55.98064990174492, 54.22845406048537, 59.96102199723095, 45.14775305242426, 38.08278812241456, 26.4475595176922, 47.09048101394354, 54.33682950456132, 60.266876608477126, 17.925745621778283, 27.612025597506335, 66.01208476754456, 36.35070830429158, 28.64271991347884, 41.906042623674686, 6.92577209468097, 4.756416253548863, 71.1424279320423, 24.90029251979333, 37.789179175198605, 41.76278378030956, 47.48131534864946, 40.765022589464095, 51.01164393154166, 2.5243786951569143, 3.663312728829526, 50.666222057377915, 66.70357709727263, 35.9007802025535, 65.34197171185149, 35.308477626117714, 33.970029190498096, 65.00544712770774, 30.40018420059492, 18.25811707908801, 18.006637603231482, 115.6250597450168, 57.56871958045248, 40.52400872882455, 55.12481889344275, 70.51399759360464, 42.71600104395106, 45.18176454543708, 29.61101797168633, 29.18406793625104, 40.66527592868476, 51.02198863200574, 86.47686475783692, 32.29971952663433, 44.624028582781335, 46.762204070534395, 76.28724378331003, 78.17691697536075, 43.37977221891368, 62.457457639519816, 64.79159052329786, 73.69420443571954, 31.86754442616419, 39.25291563616291, 43.65608173099885, 60.56635765807719, 60.32786445965821, 29.984054348533313, 69.38843400541124, 76.15990293014306, 21.571823846913386, 51.969816196243976, 33.22699261311309, 29.952210099778206, 77.377758605364, 45.292870634345036, 45.974176761307, 37.87825179559877, 49.044204954093644, 45.90365732750972, 58.46294194092078, 33.500880148028926, 8.844662025291411, 43.046619407395845, 67.05908529326784, 34.255899554502925, 76.69571648502267, 3.7534261922848633, 3.24285219428403, 37.51912308011637, 37.44122879503404, 44.668764793259555, 102.90162425573551, 93.09121961037422, 35.17052883197121, 86.42804097454582, 108.85023984453572, 61.199406421769304, 105.24962614716658, 62.73617537017257, 33.78441808952682, 42.74728019319071, 75.15320131569496, 4.189319072249255, 3.927835161237101, 32.37498045473967, 78.42650544200487, 54.76905944115858, 64.98468737221339, 50.88557741632449, 78.88931548131244, 50.475278854201534, 59.33626835513921, 27.503686269533176, 93.22956196148988, 41.48721402349351, 59.1637742554141, 28.7195775896985, 32.2467451925574, 38.58120682402671, 45.712486201278466, 37.44810614148499, 38.701059304034125, 40.14373622363226, 92.61803304130346, 44.90978768892616, 40.38447064912167, 67.64751181243984, 106.40254878170333, 56.70843549749665, 31.113003794585566, 48.83910760876901, 35.56485333831165, 129.79800071438575, 51.3249796300099, 54.01921724513272, 59.84926770968971, 49.94180298930189, 52.08143285130201, 75.91543345049625, 69.39297363043558, 42.71976418752293, 30.4817807002806, 53.881264654128934, 93.02102117213097, 39.755210935301754, 34.54220892565841, 57.13699865912708, 29.6964864108742, 63.27620601194618, 86.9846980905591, 18.34935087924229, 21.134384003853476, 58.010209752662874, 51.72190741388189, 42.5661183684958, 34.60876916111906, 66.42020680654767, 77.8493632661528, 52.92275985081488, 41.66399993278567, 121.70546975166685, 66.44484397369015, 30.001407024696242, 59.031529231492726, 101.4505102370822, 55.950762458825906, 57.39757840979072, 108.53785856549526, 61.71528861262238, 70.64177569229884, 72.8942702607838, 47.51363108644274, 51.58482696194417, 60.25357389759485, 53.92607826629941, 54.32796438118002, 78.51543069952892, 41.24285525379992, 118.25313765635757, 34.89453758977332, 64.49108473826476, 46.43748934395381, 40.149589834909875, 46.797420827599154, 56.51326657402405, 58.386313755791974, 45.14706169678635, 153.64887382683335, 48.42264299229815, 40.24886054700705, 82.76267955415362, 50.534230739302444, 44.994268987489875, 97.45154228527319, 42.71201673671736, 109.32156941215018, 60.484603148897335, 59.678011963506364, 92.17779543318872, 57.05876892991515, 121.8600842604611, 52.14405640312545, 53.834174854463726, 70.39550522057641, 36.659554838558364, 96.10474873961299, 66.59734615448679, 39.45068520805263, 62.70572319316123, 6.329177176437802, 6.476946945219192, 145.03220732522192, 74.85299378951368, 72.50452947575047, 47.20844396511566, 139.30513454260063, 67.98563161722811, 104.10976825907225, 50.45245931550968, 120.13292963316985, 62.744961168271765, 62.721454999187955, 101.95128339798225, 29.93034672542026, 78.03728472323878, 89.78412051368964, 64.0516885524462, 49.11432388575731, 51.27957160682036, 75.12676772994412, 65.56102298260991, 58.12887700914947, 49.32096492097976, 76.4382923163921, 47.33131512246857, 79.33853093880316, 42.643632771916174, 107.27359953120546, 55.67539645366452, 130.36352537080606, 69.81163482119311, 31.662545415268937, 108.70291730280212, 81.97262108168516, 80.12994072330768, 73.93150857073913, 54.935144676777725, 95.7086864285411, 78.14230158700035, 43.968743739718796, 63.09535274515713, 44.7760617160659, 70.02572975088067, 100.1643547250202, 38.408410465670734, 45.770907736859535, 52.7038329092008, 43.70216848285423, 66.35264083060724, 50.796157071578776, 40.790392259198, 36.96434908309831, 53.07948966479391, 67.00871207607017, 63.22164536191822, 71.97166645352469, 52.56434855551513, 67.59837362826448, 49.692929149059246, 53.02914372848243, 65.64409661704158, 284.84119588593626, 125.91752440519834, 101.4480592131335, 59.08051195304963, 50.89547478318874, 96.9485394212511, 102.25335212082545, 53.04875410435589, 58.89415545849081, 141.7754565092347, 54.04593810751565, 35.423927238302994, 36.31909383760186, 45.463548817235235, 123.52139688045445, 50.323156146629074, 49.41100945831436, 69.32227653704038, 40.63536481766714, 72.01398857981718, 105.51528034082335, 87.1087401274985, 46.079322046972884, 48.5413564253729, 69.07452972903556, 35.90608897790386, 60.779126747717456, 47.06782918056789, 36.21118471550566, 67.09700912475923, 129.8821293170912, 145.23263999279746, 85.6292478427136, 50.75489790897894, 47.23307155856286, 60.171363862298975, 58.97809453764742, 65.1826956611431, 72.59826112109856, 43.16630634774609, 57.98389512683075, 136.15701453036058, 104.12230112640367, 104.99528993046046, 53.53927135658367, 60.33768979292422, 56.334228115131225, 53.53923964719637, 46.572829380881515, 53.507734950486004, 64.38886542138849, 43.526388920792975, 63.28348313137006, 42.062263305447765, 67.64698730513695, 68.71457917186238, 44.319364193116684, 45.47267989457632, 47.99168238093485, 56.04017869349102, 41.00943298870175, 59.64251608379936, 57.493347939535795, 42.29583694526488, 65.75428770226904, 68.03409228756809, 57.51813165034881, 64.72746898115064, 53.10059898486605, 48.01402274288117, 48.19372294571946, 184.36584870490552, 37.14168513307585, 73.27948493892488, 41.874745534190325, 59.97239712566886, 37.0293449581523, 56.66357658193287, 136.8007247136354, 57.04410775008718, 68.43183606744206, 45.434965842792494, 50.09299985679515, 104.88939143750581, 45.8376012144737, 71.01641666099692, 51.741089484087325, 101.91714992484741, 40.78386573337541, 44.44517418802956, 44.55654534787316, 89.65453318072707, 39.72278498325569, 48.254860312571545, 37.272267355782816, 54.68565097146769, 36.65130972641563, 53.285351298831394, 60.03789398996651, 140.2308059227309, 38.19780298550498, 56.00524210182344, 47.4112286727532, 42.74135269121902, 62.15874597983325, 148.55484259751907, 40.8148875492246, 51.61884686156763, 79.97413581004902, 74.32789327603649, 55.94771294355216, 46.06115054728338, 60.13565262596347, 118.38680538539656, 100.88289623223942, 94.1809597104529, 49.724119493905526, 69.2957418040304, 88.1032301446121, 54.21208624905548, 181.89293097693718, 85.85603995123044, 78.68254317465805, 98.22425367031816, 75.52399428844765, 53.909756599553575, 81.05288412022658, 143.49591251313905, 55.78904868839752, 54.195044901484245, 60.52217698615456, 42.26769149817363, 41.25455838933076, 43.362173881475954, 103.92629242905349, 66.15813518499286, 47.50307012293049, 50.325544857009845, 46.092648872235415, 8.843269689085448, 8.96091611835778, 62.54183918214836, 86.2605434319045, 64.9618983856261, 93.12056865562968, 51.36575477299555, 129.49610813706056, 36.74391200778379, 65.29742654381387, 105.99574395992835, 57.5278570980066, 212.18765003676168, 57.64505426665399, 208.57095953529506, 49.66430680071346, 46.01123773866402, 81.72600836799045, 102.80517859759631, 35.810175882827345, 113.88550178893959, 65.13638140151372, 59.33593212658502, 54.02609068766894, 57.02455112410554, 56.59325110242183, 46.95910878209312, 87.20655196797317, 60.41825984570725, 46.24002078889759, 42.389600165316345, 79.65663119032253, 60.35149187730051, 292.910703090919, 41.758870707526455, 80.78007096928916, 165.62006012558348, 70.03261284975679, 138.40834766372154, 55.37800289313476, 73.851735833722, 50.97949371269575, 69.3101204152661, 50.82455358220701, 47.258681873430724, 94.93211364916698, 90.41534279966818, 56.04467817367912, 65.53266824667287, 57.08555398296548, 127.43380519458997, 93.61459687040887, 49.81502477415562, 55.248597682445116, 43.877045774026584, 253.2317427467283, 88.79067494985298, 42.53672576509481, 45.85445054457153, 54.00486110083755, 75.76052833320537, 52.65787539511238, 65.25280465239175, 63.5592917426385, 131.49585630745386, 165.52730192228358, 51.36871609684751, 69.99521072531142, 48.95099529649517, 71.53618515627193, 91.13570369770848, 61.490272276364585, 47.33119186006423, 55.82724708691008, 119.17589204271982, 61.33737905925632, 43.26010863041371, 55.81346084713185, 81.84236171148834, 57.67734198821673, 63.86590970790893, 54.72807431762795, 64.58977654131637, 149.16671288786253, 45.52192486422122, 74.80862818338882, 122.00028747037803, 37.880689241232545, 48.826759131698466, 71.81648991465057, 74.69780862067229, 64.7850157988409, 57.230184318461504, 131.23691921264512, 197.6966691330045, 71.7731039852503, 120.19249016641938, 55.2986503724896, 116.30291296106813, 54.700475165915954, 37.239997185455806, 65.75808984879741, 87.94350706501237, 63.69235923967002, 55.82635655868136, 52.83758697445464, 75.93834375452435, 182.19711571775773, 45.79851737851689, 79.71172700856121, 47.408835099622124, 54.62861210720974, 140.51025685059642, 58.46771087789508, 69.92542752661433, 94.97822514683142, 53.50559777301914, 50.68699615011494, 149.5686543624237, 55.176303702904214, 66.63044931672468, 89.91579425158959, 58.80849675592955, 79.91607352758442, 125.56406271789173, 47.07415876637026, 121.29123346815021, 69.06699397264786, 77.0898250540969, 62.4421859138575, 73.38529100434472, 42.072921633801016, 66.54511057602848, 169.304767403708, 100.34614015901735, 83.40066041121202, 228.82278541645934, 96.90260235588711, 64.65707674421823, 68.22323655513463, 64.00480342220699, 53.189940188482794, 44.539142543656986, 71.2756747106764, 47.50502535414573, 48.56995218904007, 54.35311822299845, 132.77801934417482, 58.41396092447509, 54.74926165197718, 52.75552178055863, 74.71978302432903, 108.38674206525329, 67.23716039667138, 71.83536469795811, 67.84526299012757, 69.05232087227945, 84.12063993736649, 65.56649486896822, 55.7758422869668, 285.31323062030623, 69.8214977167811, 163.04705429728813, 85.29820327234363, 46.38899536598117, 102.39015778291433, 125.49624407071983, 40.58732965473127, 47.02816137371356, 6.516662555567857, 7.148574959809653, 127.75287305582829, 58.12851848187766, 84.92768522762377, 55.22275187509618, 46.561075998304915, 38.77146559686882, 49.681769016194075, 73.05458334736727, 41.86524989799117, 50.805527557921636, 87.94979967518478, 67.63887435345454, 39.75276622785734, 40.52077154794485, 47.32174534156859, 130.40904614493462, 61.77016758273812, 60.720348611064175, 120.54925154426282, 77.65395524979296, 43.752788654714344, 53.577643214742224, 42.910715079311984, 179.28026073554796, 107.87103026426446, 116.77834519657743, 79.13237892170574, 102.0655292061958, 131.59156214125633, 185.07317968097368, 77.6610048682614, 76.9446771997737, 77.26583306760419, 40.47761905029661, 44.68858615075849, 53.879830482435196, 75.34965842938956, 143.50682530535659, 107.1611832962629, 98.48113247127827, 43.307600148713796, 223.72084161217475, 42.653068498291645, 97.15790126008542, 56.819124297001096, 120.70345306489904, 65.9070374171247, 59.37063351473535, 69.5106826121268, 41.557283740494945, 72.69950617739235, 34.188828145374785, 70.17641948556644, 76.04430973746403, 186.27506598388206, 108.76644987237715, 44.780023571991, 73.23161719890857, 66.87735811605695, 58.232700179563416, 72.18689907665056, 61.22704201265133, 40.966635391979345, 200.13503876291352, 26.04714658860759, 29.00730733124971, 48.52770571662195, 112.32026537254998, 80.46060998888747, 33.430205978086725, 56.70036976235504, 82.69728775693694, 168.1965439126936, 43.502441738724, 243.9543232494278, 103.86616684905947, 65.02032747330064, 49.74677992515105, 54.22172513414795, 58.79134690965491, 77.16229500698734, 53.01648125374796, 175.4960806297555, 56.33902033626501, 80.45459097651468, 60.11172133280108, 43.99677485009735, 66.6268196382155, 128.55232311203298, 38.10862910680059, 79.64531067247611, 226.18893109097795, 86.10352387917712, 58.81604691338149, 75.36943970445704, 53.37658037103435, 38.093367093919895, 85.52546161923476, 94.47555158529916, 91.54838399518157, 137.4148725209827, 128.2973471559382, 56.28120869817617, 107.11149849320122, 49.56702212223169, 114.57083136344916, 185.48589845713653, 106.76889279491837, 95.53392387035805, 52.4929645984606, 48.39367698668852, 82.26281837462196, 91.75235362441737, 58.10660915744971, 64.69507369129356, 63.63677672670407, 143.576445097999, 95.94356809980559, 96.44258392624137, 68.30206101457054, 47.4153429134311, 70.48251815271693, 35.87171481983189, 116.0926468636558, 39.38859873361373, 34.02505815242955, 38.65829816094157, 49.517472321707025, 42.155302384642475, 39.470788503992814, 41.47973385219429, 86.68163143115095, 68.05327469267067, 44.98876689580759, 58.409189934243834, 88.12743288271355, 11.531414872555963, 12.188768188488433, 59.13249259660658, 141.56734201942925, 98.97425179087172, 74.53389621983801, 89.17247176727874, 67.1582951101976, 71.05652134367503, 77.35379088471788, 6.623362858601155, 7.08377914290068, 252.55267866824582, 44.46398785228974, 133.45106961449875, 76.88366207875788, 76.07706458770846, 64.69654583519568, 63.99050440144294, 67.90432773884113, 67.1589830673004, 62.15835138996307, 72.4680602470305, 49.70585967920155, 58.23172252939515, 155.23727942808966, 183.70176949485196, 122.47392052036822, 102.93891934025498, 70.52919355026354, 79.07903412001782, 73.32654536775175, 52.84089053163371, 57.81765661981244, 39.38462185553036, 109.4584650568114, 104.6856004541253, 66.74102153743604, 110.03075082728998, 87.05003666666693, 162.51291337275273, 51.492382008624816, 63.55690479622041, 104.75130979686304, 94.31223627291783, 99.78283829019352, 154.3177990126135, 75.27153258211928, 74.02872631896517, 142.3444613090249, 75.40899274174495, 48.49868817444872, 93.47320626504566, 128.14435853128302, 41.19771191245928, 113.46788201569085, 75.22082579574845, 124.76442266092101, 45.32511724669849, 70.67490860444303, 281.18017323512663, 34.51377632188317, 54.66950251438508, 32.97150778983038, 49.4132479797052, 58.416793152363205, 167.97194964807844, 43.39631520775187, 45.042145622964334, 54.75272938791145, 57.27114427850632, 69.7933082185274, 108.45873153674005, 61.9914320515722, 55.618456720066675, 66.55554545274053, 97.28030150462286, 41.43958467749632, 5.457391684480388, 6.162854803833162, 54.87163623971265, 109.37446576925186, 38.80805718420382, 37.72975246948179, 48.32133203809874, 35.79222459680228, 75.07988065488054, 54.109139613032866, 115.88857862661102, 94.25730118145557, 62.08896579558868, 67.97220401434714, 54.595579340028195, 85.32579817495856, 67.04546771743826, 53.96842758163403, 56.35745839676873, 63.88264544328276, 116.24363529084496, 55.83838205631463, 94.59926454232333, 65.34838777227552, 170.0455980484731, 71.27532275825327, 96.74996701075112, 62.53150312749567, 217.25062072242864, 51.34772985632089, 101.2300772306903, 46.64067812835043, 85.87260379838028, 95.3690806877946, 48.68012685575883, 93.4941975285556, 30.57518562886195, 46.426412216318404, 86.18424099398216, 61.469557438584424, 243.7224035396157, 68.27828822935714, 91.84056637873373, 15.223438241238526, 12.666001957991726, 35.85006453019039, 76.63486244407066, 76.86974368049565, 60.406424841204235, 45.52798072399692, 87.67450970702814, 71.01283872021932, 47.04440914647914, 91.06604453481116, 75.50994392718368, 127.63903823968987, 94.69111267902397, 246.57760170556088, 59.00368955494988, 90.06996765528002, 49.651826756323175, 59.67328645444585, 109.29382130116096, 143.18791330008082, 115.33868316010465, 58.15485749929042, 56.50896216960032, 122.62253809297708, 102.37498847143239, 70.78528091652191, 134.35015717785558, 139.92362927684587, 173.24435531647555, 56.39676099764107, 85.98662456548465, 105.758465718937, 55.09811403783638, 103.11275553172857, 49.18315946913488, 65.58341978779353, 71.31221756152004, 60.874160827612386, 46.95083882277269, 92.7267524509579, 69.67878993878082, 47.8327163956097, 49.174131956995694, 69.28984881925155, 81.58698930904315, 40.96643744618771, 116.37912346524043, 112.26934774640111, 142.75619263203555, 61.26570780385023, 78.31157841636168, 64.67437872635693, 44.895994918728434, 98.5898803031006, 128.99209033141062, 44.53733895005189, 82.48358460264886, 90.82103679469756, 39.3768974909712, 84.94935108210393, 63.0084856309972, 100.06136483497514, 86.8068904579816, 198.7869029027234, 48.93948761759872, 98.33392434721266, 47.396401632926384, 75.56256092315374, 43.797922883248, 73.91157298403218, 77.30578265809694, 80.23505224676566, 79.65372862153295, 105.72751951922952, 34.22331179067877, 88.42689613360946, 41.44576922143109, 66.32121509616844, 50.703600695751646, 69.31715058959975, 60.96654195635117, 85.80748437507862, 53.41456918173279, 104.2386753516907, 100.50334267365959, 101.44378026785267, 79.81093588296804, 88.46946230700576, 215.08908520158369, 80.53182117142413, 109.86294287154203, 152.66326362147146, 48.49740712417788, 70.3072479943913, 49.06582886267901, 78.93878168266176, 118.79471030274007, 43.48435262821008, 70.17409235642984, 77.92400547712468, 67.42074935196173, 120.44931404604327, 139.6451902936253, 77.8505136085281, 92.62948731388175, 75.9028852023425, 70.0194260055903, 142.5867585843633, 42.695988314519674, 62.623771753663746, 46.77366151448337, 65.89839144370123, 153.18362855775203, 56.78327576601021, 87.82033184708642, 67.21710867599045, 135.23777946549873, 102.70263814066651, 74.24674172826232, 116.37888065343648, 77.62722443789853, 119.57168152461128, 54.3731677562662, 81.19827858658005, 96.32073801689343, 232.0260644657611, 53.24630947551673, 200.3326409607819, 9.822570041466745, 167.05880316115798, 59.28048353115517, 130.13239872268534, 90.86094358756785, 46.426738869753486, 57.181418571999366, 204.97007996678914, 77.31928405563544, 43.46566076246486, 126.96760973404538, 101.9443584877875, 65.92105877430227, 57.14744712849187, 71.75081275775295, 80.51919105740161, 142.1068229072155, 55.04731551094081, 85.80310313394419, 101.35948886811568, 70.3990492442267, 74.48938683989319, 261.3826695234104, 99.10145004581996, 114.47774228498544, 192.78888697974176, 104.31119045013403, 86.40235988667047, 82.77092817592748, 134.21062107204645, 119.38837011365354, 44.800051146673525, 171.20956509580438, 149.69856559895834, 90.98379866667482, 81.58084284474026, 94.17283785448075, 510.6402459689766, 99.59621570134101, 88.8982843499641, 71.94080971025471, 131.72957675523057, 85.30110567088747, 62.20292015314045, 75.30368878114825, 110.37485212235312, 107.4185079563217, 76.44050979348143, 37.528930493993755, 89.28553407470345, 82.18882695624296, 120.08596510830883, 61.81503414956561, 71.43154992590195, 78.49027825495472, 96.75609862801285, 67.45385233437568, 103.44416389229701, 81.67705412108982, 98.13886269754128, 108.71372389102777, 67.10420557644026, 50.85199933638067, 54.02373427612682, 82.41568895793502, 45.230058363809704, 75.98450113541669, 94.74709408988252, 60.46659984316816, 76.99287469159827, 69.02406805711526, 39.82710440895492, 104.7513335218378, 72.52695403915094, 56.202991558542834, 66.86925189238136, 121.33056600128654, 65.87821118601407, 277.8281206907003, 66.38821332233157, 83.56214254521393, 51.12646895538518, 262.30289592326847, 74.51249602789609, 98.02537970006047, 66.32404473851312, 38.28043226169786, 78.53200016192645, 80.87834516119015, 123.03606004924883, 58.53726901164892, 43.4188078573685, 85.8919082239216, 167.10860639221386, 42.68244840153561, 39.04460898548951, 145.40092965374268, 94.1295257889872, 34.09996835716792, 169.2332433959068, 77.6074169158557, 41.386553462573545, 116.1931095584755, 123.19827739658244, 73.72082807669351, 72.23730191180252, 285.88662892415283, 84.07156656887176, 120.46056209172707, 47.38618099277747, 60.637777157917746, 192.576646420112, 80.71002084505162, 146.22317734856085, 66.69072770167895, 59.89006496139769, 132.10599299190886, 46.12381460568322, 65.22281714292582, 129.5389517496332, 151.5664910401468, 92.49623235683458, 92.44357062031564, 55.749826949973155, 69.63942037030394, 84.42193917158504, 53.349362579149016, 54.51175120338381, 71.18382769528976, 66.96345186222179, 78.66524925640466, 193.02128865407425, 258.0385167407758, 88.95674108719074, 40.68135577397964, 84.8001953217157, 63.18324256790416, 49.5491806870792, 129.26608237049714, 69.74290667551638, 45.487672107087434, 59.21690189607198, 97.7933623858174, 135.00123723558482, 46.56611887266744, 41.520874995184634, 51.78333352209553, 87.12770243795853, 28.427123117539406, 160.1036608434883, 111.16784601364044, 124.78824587277755, 44.29400631687818, 149.73743441787101, 69.96010076300217, 151.62213715163372, 93.47265097783219, 41.019484088549326, 57.999705395065156, 41.23958353951462, 139.81589909049308, 39.60460659143582, 144.67411149345256, 68.92832514905125, 73.15176818397325, 88.78161790061311, 116.7949358469485, 81.63330174223589, 54.49602075937425, 150.1347118324538, 108.37445934366603, 81.78521911713129, 48.17034743109992, 171.71879651337943, 75.05927111210647, 116.71376285852753, 189.53195705383078, 55.631778112951984, 92.6163732735184, 79.60537528352059, 50.27213042573391, 73.83818671692487, 98.60403376168888, 50.64782917804883, 157.00701711684258, 143.1170939846712, 73.62889965920539, 43.847015079256664, 113.69314435598379, 50.37572495706002, 114.46411483513812, 45.10640216575663, 70.9967640755029, 183.92041355074738, 103.75383191472929, 73.2107507330122, 88.19856207753453, 94.69980848120251, 130.0275726519299, 91.4870320851146, 208.2605092155607, 61.607319358519355, 252.08170641691996, 63.64263373617923, 192.79544999819834, 81.29694283184106, 123.98131209164586, 45.099351009728096, 55.43455563386443, 45.70551496896499, 97.82902345337699, 59.19488221614585, 126.9033271620922, 84.57940035090645, 87.3123647456313, 138.37699885043497, 73.95962845281582, 43.44424936816832, 105.87308030242633, 7.851702475355082, 8.932386189588163, 60.85416313650693, 58.35966023754927, 178.83836952947763, 67.82005661414068, 54.622925440452796, 286.0306396159791, 122.51872089313444, 190.03070903046358, 78.46306431924035, 98.45453105052931, 13.1136635864336, 13.501563696124023, 65.3507172016375, 88.48485307525291, 121.50133005805085, 145.4183780926679, 178.74899076579112, 98.15396675466565, 93.8727578781647, 53.4230997843519, 47.52892247194773, 73.28392762867225, 40.37609278621196, 147.16988375984343, 106.04833893931696, 84.14678359542698, 71.31860270410922, 108.26014670942683, 187.60445358923113, 75.3044385779144, 65.49180883351166, 51.06347234465788, 45.460709081764875, 77.55522291943478, 51.27253828944625, 86.04732090394285, 45.85549234435291, 45.46721510516743, 55.39407996851434, 77.79010008422111, 90.34625623994987, 140.695790825201, 104.92194055773422, 198.12861469757314, 33.90082211577253, 51.518211073407315, 95.20399718252423, 106.7279471084375, 73.30830010758842, 254.21849148672493, 97.26528839589331, 145.7082170699157, 95.20738341436615, 22.384867148611953, 23.269770104500694, 102.81659984826709, 46.69084073359076, 71.82014632925801, 82.01752656318986, 32.62650554790432, 163.01326615022256, 36.305398747314186, 10.245543972428187, 9.693697211658565, 128.87189890667742, 37.271775765152476, 76.82576973551201, 56.44204420769854, 110.33938966890261, 96.87162963316794, 195.93342843667259, 68.22216503192247, 112.55504751320815, 94.39232937668568, 75.00163885678371, 225.81802929834316, 49.63175840125541, 62.572766158957364, 109.16615019050198, 132.654791</t>
         </is>
       </c>
-      <c r="R9" t="n">
+      <c r="R9" s="3" t="n">
         <v>123.3914333343506</v>
       </c>
-      <c r="S9" t="n">
+      <c r="S9" s="3" t="n">
         <v>57.51475047808284</v>
       </c>
-      <c r="T9" t="n">
-        <v>10</v>
-      </c>
-      <c r="U9" t="inlineStr">
+      <c r="T9" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
         <is>
           <t>[120.61085510253906, 147.2869110107422, 50.89359664916992, 196.46749877929688, 65.52867126464844, 219.75584411621094, 39.56925964355469, 126.93525695800781, 165.2930908203125, 101.57334899902344]</t>
         </is>
       </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>p-1.0shalton2118</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:21:11</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4096</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ppo</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>100</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.183065603014852</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.5211024971331032</v>
+      </c>
+      <c r="N10" t="n">
+        <v>106.2631578947368</v>
+      </c>
+      <c r="O10" t="n">
+        <v>38</v>
+      </c>
+      <c r="P10" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>[1.0279017306107405, 1.1069428575895663, 1.102887579488172, 0.5255031190730329, 1.8556245880033027, 1.3473975718733877, 0.5094010216220801, 1.7022731783341198, 0.6029745261802829, 0.4281843647253538, 0.7760156169209359, 0.6110677948885319, 1.878591349846404, 2.331854910164841, 1.2721659274641721, 1.6665073055734767, 1.19079453691316, 1.464521078238047, 1.3793445426293414, 1.9345053887238055, 0.926109334437943, 0.3705093887164873, 1.4854944139683282, 1.416748887243379, 1.053260340917286, 0.37237557739556115, 0.5768926841260956, 0.9320532799114819, 0.7844862921441665, 1.539989444796599, 0.921544514320304, 1.4478690084925143, 1.4947647210894344, 1.0060356579060168, 2.3828062964098375, 1.0885134098357379, 1.7405196222649206, 0.7020610517255315]</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="1048557" ht="12.75" customHeight="1" s="2"/>
     <row r="1048558" ht="12.75" customHeight="1" s="2"/>

</xml_diff>